<commit_message>
Add more products into cart
</commit_message>
<xml_diff>
--- a/Config/TestData.xlsx
+++ b/Config/TestData.xlsx
@@ -1,32 +1,22 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Playwright setup\AutomationExercise\Config\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45147740-09EB-46EF-9213-44B375F39A6B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" activeTab="1" xr2:uid="{52D6294C-7B91-43C7-94D4-3EE66AA36EE4}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8364" activeTab="1"/>
   </bookViews>
   <sheets>
-    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
-    <sheet name="HomeData" sheetId="2" r:id="rId2"/>
+    <sheet sheetId="1" name="LoginData" state="visible" r:id="rId4"/>
+    <sheet sheetId="2" name="HomeData" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="ProductData" state="visible" r:id="rId6"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-  </extLst>
+  <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>username</t>
   </si>
@@ -44,27 +34,42 @@
   </si>
   <si>
     <t>https://automationexercise.com/</t>
+  </si>
+  <si>
+    <t>ProductName</t>
+  </si>
+  <si>
+    <t>Fancy Green Top</t>
+  </si>
+  <si>
+    <t>Blue Top</t>
+  </si>
+  <si>
+    <t>Men Tshirt</t>
+  </si>
+  <si>
+    <t>Stylish Dress</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
-      <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
     <font>
       <u/>
-      <sz val="11"/>
       <color theme="10"/>
-      <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
@@ -84,16 +89,14 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -405,14 +408,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F66F328B-7310-41B2-B9FF-CA6DC5BC3D38}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
     <col min="2" max="2" width="25" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -420,7 +423,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -430,21 +433,21 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1" r:id="rId1" xr:uid="{B0971DBA-D3D5-49B1-B518-D5ADA19DBFFC}"/>
+    <hyperlink ref="B1" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{788BFCF3-4A93-4C43-BEC2-35379B2153FB}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0.3" customHeight="1"/>
   <cols>
-    <col min="2" max="2" width="28.77734375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="28.77734375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -454,8 +457,44 @@
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B1" r:id="rId1" xr:uid="{91CB0C11-B0D4-468F-B166-AF34DA575093}"/>
+    <hyperlink ref="B1" r:id="rId1"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:A5"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
+</worksheet>
 </file>
</xml_diff>